<commit_message>
#5 Client BOM update.
@basit-eSpark  R21 ko DNP kr dia ha BOM me 10K Wala.
</commit_message>
<xml_diff>
--- a/Design-Files/Audio-Player-v1.0/Deliverables/BOM/Client-BOM-Audio-Player-v1.0.xlsx
+++ b/Design-Files/Audio-Player-v1.0/Deliverables/BOM/Client-BOM-Audio-Player-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="215">
   <si>
     <t>#</t>
   </si>
@@ -658,13 +658,19 @@
   </si>
   <si>
     <t>Custom</t>
+  </si>
+  <si>
+    <t>R21</t>
+  </si>
+  <si>
+    <t>DO NOT PLACE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -703,6 +709,22 @@
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -823,7 +845,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -862,6 +884,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1150,7 +1181,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1162,7 +1193,7 @@
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1246,7 +1277,7 @@
     <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B44" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B45" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -2173,385 +2204,416 @@
     </row>
     <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
-      <c r="B33" s="11">
-        <f>ROW(B33) - ROW($B$2)</f>
-        <v>31</v>
-      </c>
-      <c r="C33" s="12" t="s">
+      <c r="B33" s="11"/>
+      <c r="C33" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D33" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="F33" s="7" t="s">
+      <c r="D33" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="E33" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="F33" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="G33" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="H33" s="7" t="s">
+      <c r="G33" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="H33" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="I33" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="J33" s="7">
-        <v>4</v>
-      </c>
-      <c r="K33" s="7"/>
+      <c r="I33" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="J33" s="15">
+        <v>1</v>
+      </c>
+      <c r="K33" s="17" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B34) - ROW($B$2)</f>
         <v>32</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="F34" s="9" t="s">
+      <c r="D34" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F34" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="G34" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="H34" s="9" t="s">
+      <c r="G34" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H34" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="I34" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="J34" s="9">
-        <v>2</v>
-      </c>
-      <c r="K34" s="9"/>
+      <c r="I34" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="J34" s="7">
+        <v>4</v>
+      </c>
+      <c r="K34" s="7"/>
     </row>
     <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
-        <f>ROW(B35) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="H35" s="7" t="s">
+      <c r="D35" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H35" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="I35" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="J35" s="7">
-        <v>1</v>
-      </c>
-      <c r="K35" s="7"/>
+      <c r="I35" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="J35" s="9">
+        <v>2</v>
+      </c>
+      <c r="K35" s="9"/>
     </row>
     <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B36) - ROW($B$2)</f>
         <v>34</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="H36" s="9" t="s">
+      <c r="C36" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="H36" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="I36" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="J36" s="9">
-        <v>1</v>
-      </c>
-      <c r="K36" s="9"/>
+      <c r="I36" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="J36" s="7">
+        <v>1</v>
+      </c>
+      <c r="K36" s="7"/>
     </row>
     <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
-        <f>ROW(B37) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C37" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="H37" s="7" t="s">
+      <c r="C37" s="13"/>
+      <c r="D37" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="I37" s="8" t="s">
+      <c r="I37" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="J37" s="7">
-        <v>2</v>
-      </c>
-      <c r="K37" s="7"/>
+      <c r="J37" s="9">
+        <v>1</v>
+      </c>
+      <c r="K37" s="9"/>
     </row>
     <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B38) - ROW($B$2)</f>
         <v>36</v>
       </c>
-      <c r="C38" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="I38" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="J38" s="9">
+      <c r="C38" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="J38" s="7">
         <v>2</v>
       </c>
-      <c r="K38" s="9"/>
-    </row>
-    <row r="39" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K38" s="7"/>
+    </row>
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
-        <f>ROW(B39) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="C39" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>99</v>
+      <c r="C39" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>98</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>174</v>
+        <v>123</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H39" s="9" t="s">
+        <v>182</v>
       </c>
       <c r="I39" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="J39" s="7">
-        <v>6</v>
-      </c>
-      <c r="K39" s="7"/>
-    </row>
-    <row r="40" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J39" s="9">
+        <v>2</v>
+      </c>
+      <c r="K39" s="9"/>
+    </row>
+    <row r="40" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B40) - ROW($B$2)</f>
         <v>38</v>
       </c>
-      <c r="C40" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>100</v>
+      <c r="C40" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="G40" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="H40" s="9" t="s">
-        <v>183</v>
+        <v>212</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>174</v>
       </c>
       <c r="I40" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="J40" s="9">
-        <v>1</v>
-      </c>
-      <c r="K40" s="9"/>
-    </row>
-    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J40" s="7">
+        <v>6</v>
+      </c>
+      <c r="K40" s="7"/>
+    </row>
+    <row r="41" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
-        <f>ROW(B41) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="C41" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>184</v>
+      <c r="D41" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>183</v>
       </c>
       <c r="I41" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="J41" s="7">
-        <v>1</v>
-      </c>
-      <c r="K41" s="7"/>
+      <c r="J41" s="9">
+        <v>1</v>
+      </c>
+      <c r="K41" s="9"/>
     </row>
     <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B42) - ROW($B$2)</f>
         <v>40</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="G42" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="H42" s="9" t="s">
-        <v>185</v>
+      <c r="D42" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>184</v>
       </c>
       <c r="I42" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="J42" s="9">
-        <v>1</v>
-      </c>
-      <c r="K42" s="9"/>
+      <c r="J42" s="7">
+        <v>1</v>
+      </c>
+      <c r="K42" s="7"/>
     </row>
     <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
-        <f>ROW(B43) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="C43" s="12" t="s">
+      <c r="C43" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D43" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="G43" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>173</v>
+      <c r="D43" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>185</v>
       </c>
       <c r="I43" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="J43" s="7">
-        <v>1</v>
-      </c>
-      <c r="K43" s="7"/>
+      <c r="J43" s="9">
+        <v>1</v>
+      </c>
+      <c r="K43" s="9"/>
     </row>
     <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B44) - ROW($B$2)</f>
         <v>42</v>
       </c>
-      <c r="C44" s="13" t="s">
+      <c r="C44" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D44" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="G44" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="H44" s="9" t="s">
-        <v>186</v>
+      <c r="D44" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>173</v>
       </c>
       <c r="I44" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="J44" s="9">
-        <v>1</v>
-      </c>
-      <c r="K44" s="9"/>
+      <c r="J44" s="7">
+        <v>1</v>
+      </c>
+      <c r="K44" s="7"/>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="1"/>
+      <c r="B45" s="11">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="H45" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I45" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="J45" s="9">
+        <v>1</v>
+      </c>
+      <c r="K45" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>